<commit_message>
Mejorar diseno visual de figuras ROC, Precision-Recall y Calibracion para publicacion Q1
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -529,10 +529,10 @@
         <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.2831490039825439</v>
+        <v>0.2218894958496094</v>
       </c>
       <c r="L2">
-        <v>0.01512765884399414</v>
+        <v>0.02072834968566895</v>
       </c>
       <c r="M2">
         <v>0.4347826086956522</v>
@@ -594,10 +594,10 @@
         <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.404062032699585</v>
+        <v>0.3529021739959717</v>
       </c>
       <c r="L3">
-        <v>0.0681915283203125</v>
+        <v>0.04961013793945312</v>
       </c>
       <c r="M3">
         <v>0.1304347826086956</v>
@@ -659,10 +659,10 @@
         <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.4068689346313477</v>
+        <v>0.3562710285186768</v>
       </c>
       <c r="L4">
-        <v>0.06644797325134277</v>
+        <v>0.0355217456817627</v>
       </c>
       <c r="M4">
         <v>0.1159420289855072</v>
@@ -724,10 +724,10 @@
         <v>0.8047587871551514</v>
       </c>
       <c r="K5">
-        <v>0.1524162292480469</v>
+        <v>0.1504209041595459</v>
       </c>
       <c r="L5">
-        <v>0.01700639724731445</v>
+        <v>0.01784181594848633</v>
       </c>
       <c r="M5">
         <v>0.5072463768115942</v>
@@ -789,10 +789,10 @@
         <v>0.969726295729061</v>
       </c>
       <c r="K6">
-        <v>0.1307473182678223</v>
+        <v>0.1300246715545654</v>
       </c>
       <c r="L6">
-        <v>0.007755756378173828</v>
+        <v>0.007639169692993164</v>
       </c>
       <c r="M6">
         <v>0.5652173913043478</v>
@@ -854,10 +854,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K7">
-        <v>0.01709771156311035</v>
+        <v>0.0109407901763916</v>
       </c>
       <c r="L7">
-        <v>0.002440214157104492</v>
+        <v>0.002017021179199219</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -919,10 +919,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K8">
-        <v>0.001275062561035156</v>
+        <v>0.001119852066040039</v>
       </c>
       <c r="L8">
-        <v>0.0002858638763427734</v>
+        <v>0.0002071857452392578</v>
       </c>
       <c r="M8">
         <v>0</v>

</xml_diff>

<commit_message>
Corregir ubicacion de leyendas en figuras PR, Calibracion y ROC para evitar superposicion de lineas
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -529,10 +529,10 @@
         <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.2218894958496094</v>
+        <v>0.2206330299377441</v>
       </c>
       <c r="L2">
-        <v>0.02072834968566895</v>
+        <v>0.01331067085266113</v>
       </c>
       <c r="M2">
         <v>0.4347826086956522</v>
@@ -594,10 +594,10 @@
         <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.3529021739959717</v>
+        <v>0.312056303024292</v>
       </c>
       <c r="L3">
-        <v>0.04961013793945312</v>
+        <v>0.04988741874694824</v>
       </c>
       <c r="M3">
         <v>0.1304347826086956</v>
@@ -659,10 +659,10 @@
         <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.3562710285186768</v>
+        <v>0.4063942432403564</v>
       </c>
       <c r="L4">
-        <v>0.0355217456817627</v>
+        <v>0.04954266548156738</v>
       </c>
       <c r="M4">
         <v>0.1159420289855072</v>
@@ -724,10 +724,10 @@
         <v>0.8047587871551514</v>
       </c>
       <c r="K5">
-        <v>0.1504209041595459</v>
+        <v>0.1659379005432129</v>
       </c>
       <c r="L5">
-        <v>0.01784181594848633</v>
+        <v>0.01733136177062988</v>
       </c>
       <c r="M5">
         <v>0.5072463768115942</v>
@@ -789,10 +789,10 @@
         <v>0.969726295729061</v>
       </c>
       <c r="K6">
-        <v>0.1300246715545654</v>
+        <v>0.1485052108764648</v>
       </c>
       <c r="L6">
-        <v>0.007639169692993164</v>
+        <v>0.008794784545898438</v>
       </c>
       <c r="M6">
         <v>0.5652173913043478</v>
@@ -854,10 +854,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K7">
-        <v>0.0109407901763916</v>
+        <v>0.01198387145996094</v>
       </c>
       <c r="L7">
-        <v>0.002017021179199219</v>
+        <v>0.002028703689575195</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -919,10 +919,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K8">
-        <v>0.001119852066040039</v>
+        <v>0.00103449821472168</v>
       </c>
       <c r="L8">
-        <v>0.0002071857452392578</v>
+        <v>0.0002200603485107422</v>
       </c>
       <c r="M8">
         <v>0</v>

</xml_diff>

<commit_message>
Solucionar de forma definitiva la superposicion de leyendas en PR y Calibracion Arma de Fuego
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -529,10 +529,10 @@
         <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.2206330299377441</v>
+        <v>0.2107272148132324</v>
       </c>
       <c r="L2">
-        <v>0.01331067085266113</v>
+        <v>0.01329731941223145</v>
       </c>
       <c r="M2">
         <v>0.4347826086956522</v>
@@ -594,10 +594,10 @@
         <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.312056303024292</v>
+        <v>0.3512656688690186</v>
       </c>
       <c r="L3">
-        <v>0.04988741874694824</v>
+        <v>0.06492185592651367</v>
       </c>
       <c r="M3">
         <v>0.1304347826086956</v>
@@ -659,10 +659,10 @@
         <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.4063942432403564</v>
+        <v>0.3473000526428223</v>
       </c>
       <c r="L4">
-        <v>0.04954266548156738</v>
+        <v>0.05013513565063477</v>
       </c>
       <c r="M4">
         <v>0.1159420289855072</v>
@@ -724,10 +724,10 @@
         <v>0.8047587871551514</v>
       </c>
       <c r="K5">
-        <v>0.1659379005432129</v>
+        <v>0.166933536529541</v>
       </c>
       <c r="L5">
-        <v>0.01733136177062988</v>
+        <v>0.01660490036010742</v>
       </c>
       <c r="M5">
         <v>0.5072463768115942</v>
@@ -789,10 +789,10 @@
         <v>0.969726295729061</v>
       </c>
       <c r="K6">
-        <v>0.1485052108764648</v>
+        <v>0.135167121887207</v>
       </c>
       <c r="L6">
-        <v>0.008794784545898438</v>
+        <v>0.00794529914855957</v>
       </c>
       <c r="M6">
         <v>0.5652173913043478</v>
@@ -854,10 +854,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K7">
-        <v>0.01198387145996094</v>
+        <v>0.01142382621765137</v>
       </c>
       <c r="L7">
-        <v>0.002028703689575195</v>
+        <v>0.002035856246948242</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -919,10 +919,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K8">
-        <v>0.00103449821472168</v>
+        <v>0.000881195068359375</v>
       </c>
       <c r="L8">
-        <v>0.0002200603485107422</v>
+        <v>0.0002133846282958984</v>
       </c>
       <c r="M8">
         <v>0</v>

</xml_diff>

<commit_message>
Ajustar leyendas de calibracion: Arma Blanca (arriba), Arma de Fuego (abajo derecha), Otros (arriba)
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -529,10 +529,10 @@
         <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.2107272148132324</v>
+        <v>0.2436256408691406</v>
       </c>
       <c r="L2">
-        <v>0.01329731941223145</v>
+        <v>0.02095317840576172</v>
       </c>
       <c r="M2">
         <v>0.4347826086956522</v>
@@ -594,10 +594,10 @@
         <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.3512656688690186</v>
+        <v>0.33992600440979</v>
       </c>
       <c r="L3">
-        <v>0.06492185592651367</v>
+        <v>0.04746150970458984</v>
       </c>
       <c r="M3">
         <v>0.1304347826086956</v>
@@ -659,10 +659,10 @@
         <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.3473000526428223</v>
+        <v>0.3677914142608643</v>
       </c>
       <c r="L4">
-        <v>0.05013513565063477</v>
+        <v>0.04904532432556152</v>
       </c>
       <c r="M4">
         <v>0.1159420289855072</v>
@@ -724,10 +724,10 @@
         <v>0.8047587871551514</v>
       </c>
       <c r="K5">
-        <v>0.166933536529541</v>
+        <v>0.1700577735900879</v>
       </c>
       <c r="L5">
-        <v>0.01660490036010742</v>
+        <v>0.01262187957763672</v>
       </c>
       <c r="M5">
         <v>0.5072463768115942</v>
@@ -789,10 +789,10 @@
         <v>0.969726295729061</v>
       </c>
       <c r="K6">
-        <v>0.135167121887207</v>
+        <v>0.1284916400909424</v>
       </c>
       <c r="L6">
-        <v>0.00794529914855957</v>
+        <v>0.008140325546264648</v>
       </c>
       <c r="M6">
         <v>0.5652173913043478</v>
@@ -854,10 +854,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K7">
-        <v>0.01142382621765137</v>
+        <v>0.01878595352172852</v>
       </c>
       <c r="L7">
-        <v>0.002035856246948242</v>
+        <v>0.004369497299194336</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -919,10 +919,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K8">
-        <v>0.000881195068359375</v>
+        <v>0.001563072204589844</v>
       </c>
       <c r="L8">
-        <v>0.0002133846282958984</v>
+        <v>0.0002064704895019531</v>
       </c>
       <c r="M8">
         <v>0</v>

</xml_diff>

<commit_message>
Agregar figuras de matrices de confusion combinadas e individuales para los 3 modelos principales
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -529,10 +529,10 @@
         <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.2436256408691406</v>
+        <v>0.2567212581634521</v>
       </c>
       <c r="L2">
-        <v>0.02095317840576172</v>
+        <v>0.01174426078796387</v>
       </c>
       <c r="M2">
         <v>0.4347826086956522</v>
@@ -594,10 +594,10 @@
         <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.33992600440979</v>
+        <v>0.3280928134918213</v>
       </c>
       <c r="L3">
-        <v>0.04746150970458984</v>
+        <v>0.0642998218536377</v>
       </c>
       <c r="M3">
         <v>0.1304347826086956</v>
@@ -659,10 +659,10 @@
         <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.3677914142608643</v>
+        <v>0.4759752750396729</v>
       </c>
       <c r="L4">
-        <v>0.04904532432556152</v>
+        <v>0.06638669967651367</v>
       </c>
       <c r="M4">
         <v>0.1159420289855072</v>
@@ -724,10 +724,10 @@
         <v>0.8047587871551514</v>
       </c>
       <c r="K5">
-        <v>0.1700577735900879</v>
+        <v>0.1455605030059814</v>
       </c>
       <c r="L5">
-        <v>0.01262187957763672</v>
+        <v>0.009238481521606445</v>
       </c>
       <c r="M5">
         <v>0.5072463768115942</v>
@@ -789,10 +789,10 @@
         <v>0.969726295729061</v>
       </c>
       <c r="K6">
-        <v>0.1284916400909424</v>
+        <v>0.1194746494293213</v>
       </c>
       <c r="L6">
-        <v>0.008140325546264648</v>
+        <v>0.00726771354675293</v>
       </c>
       <c r="M6">
         <v>0.5652173913043478</v>
@@ -854,10 +854,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K7">
-        <v>0.01878595352172852</v>
+        <v>0.01032352447509766</v>
       </c>
       <c r="L7">
-        <v>0.004369497299194336</v>
+        <v>0.002128362655639648</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -919,10 +919,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K8">
-        <v>0.001563072204589844</v>
+        <v>0.001068592071533203</v>
       </c>
       <c r="L8">
-        <v>0.0002064704895019531</v>
+        <v>0.0002553462982177734</v>
       </c>
       <c r="M8">
         <v>0</v>

</xml_diff>

<commit_message>
Completar ejecucion rigurosa de Bootstrap (1000 iteraciones) y actualizar reporte en GitHub
</commit_message>
<xml_diff>
--- a/outputs/metrics/model_comparison_metrics.xlsx
+++ b/outputs/metrics/model_comparison_metrics.xlsx
@@ -529,10 +529,10 @@
         <v>0.6583301424980164</v>
       </c>
       <c r="K2">
-        <v>0.2567212581634521</v>
+        <v>0.2755334377288818</v>
       </c>
       <c r="L2">
-        <v>0.01174426078796387</v>
+        <v>0.01671552658081055</v>
       </c>
       <c r="M2">
         <v>0.4347826086956522</v>
@@ -594,10 +594,10 @@
         <v>0.4975808672548777</v>
       </c>
       <c r="K3">
-        <v>0.3280928134918213</v>
+        <v>0.331855297088623</v>
       </c>
       <c r="L3">
-        <v>0.0642998218536377</v>
+        <v>0.04887747764587402</v>
       </c>
       <c r="M3">
         <v>0.1304347826086956</v>
@@ -659,10 +659,10 @@
         <v>0.3827449936991343</v>
       </c>
       <c r="K4">
-        <v>0.4759752750396729</v>
+        <v>0.3869502544403076</v>
       </c>
       <c r="L4">
-        <v>0.06638669967651367</v>
+        <v>0.05033969879150391</v>
       </c>
       <c r="M4">
         <v>0.1159420289855072</v>
@@ -724,10 +724,10 @@
         <v>0.8047587871551514</v>
       </c>
       <c r="K5">
-        <v>0.1455605030059814</v>
+        <v>0.2048220634460449</v>
       </c>
       <c r="L5">
-        <v>0.009238481521606445</v>
+        <v>0.01209616661071777</v>
       </c>
       <c r="M5">
         <v>0.5072463768115942</v>
@@ -789,10 +789,10 @@
         <v>0.969726295729061</v>
       </c>
       <c r="K6">
-        <v>0.1194746494293213</v>
+        <v>0.1338098049163818</v>
       </c>
       <c r="L6">
-        <v>0.00726771354675293</v>
+        <v>0.009302854537963867</v>
       </c>
       <c r="M6">
         <v>0.5652173913043478</v>
@@ -854,10 +854,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K7">
-        <v>0.01032352447509766</v>
+        <v>0.01168060302734375</v>
       </c>
       <c r="L7">
-        <v>0.002128362655639648</v>
+        <v>0.002372026443481445</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -919,10 +919,10 @@
         <v>3.366568070443856</v>
       </c>
       <c r="K8">
-        <v>0.001068592071533203</v>
+        <v>0.001213788986206055</v>
       </c>
       <c r="L8">
-        <v>0.0002553462982177734</v>
+        <v>0.0002117156982421875</v>
       </c>
       <c r="M8">
         <v>0</v>

</xml_diff>